<commit_message>
Refacored Sanity...few are left because of issue Refactored Planning..few are left because of issue
</commit_message>
<xml_diff>
--- a/src/main/resources/StrategicPlan_Field_Values.xlsx
+++ b/src/main/resources/StrategicPlan_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23001"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98B20792-6D33-44CB-81EA-51D257FC3A01}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1564C219-B6E0-42B8-B105-5F89965692A7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" firstSheet="1" activeTab="5" xr2:uid="{71FE9D5D-4309-4F80-A035-2E28B4707F3C}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="1" activeTab="1" xr2:uid="{71FE9D5D-4309-4F80-A035-2E28B4707F3C}"/>
   </bookViews>
   <sheets>
     <sheet name="StrategicPlanCreation" sheetId="1" r:id="rId1"/>
@@ -445,13 +445,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9837C433-2C9A-4F7C-97EE-1D5C997FE884}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="16.69140625" customWidth="1"/>
-    <col min="3" max="3" width="38.765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="38.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -462,7 +462,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -473,7 +473,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -484,7 +484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -503,14 +503,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FA57190-D900-451B-810A-BD57BAEC856E}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.4609375" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -521,7 +521,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -541,14 +541,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9653EDE-4E0B-4AC6-BAEF-CF93CD09025C}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.69140625" customWidth="1"/>
-    <col min="2" max="2" width="17.53515625" customWidth="1"/>
-    <col min="3" max="3" width="34.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="17.53125" customWidth="1"/>
+    <col min="3" max="3" width="34.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -559,7 +559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -579,13 +579,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99BB8A33-24B3-4864-BE50-676E7C8A1E49}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="21.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,7 +596,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -615,13 +615,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24210023-6C88-4225-A708-33A47A891615}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="14.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.3046875" customWidth="1"/>
+    <col min="2" max="2" width="14.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -632,7 +632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -652,13 +652,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02892048-8F2D-4DC2-B040-2F7DFB652348}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="21.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -669,7 +669,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>

</xml_diff>